<commit_message>
Make the year plan easier to follow and keep winter, garden, and iron feeds on the right cadence.
Split calendar and text views, alternate FFR with Activ8, add iron for deep-green lawns, and turn the product notes into a short list.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/product_usage_guide.xlsx
+++ b/data/product_usage_guide.xlsx
@@ -4104,23 +4104,23 @@
           <t>spread</t>
         </is>
       </c>
-      <c r="Q30" s="5" t="n">
-        <v>1</v>
+      <c r="Q30" s="4" t="n">
+        <v>0</v>
       </c>
       <c r="R30" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="S30" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="T30" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="U30" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="V30" s="8" t="n">
-        <v>1</v>
+      <c r="S30" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T30" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U30" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="V30" s="4" t="n">
+        <v>0</v>
       </c>
       <c r="W30" s="4" t="n">
         <v>0</v>

</xml_diff>